<commit_message>
Completar procesamiento de indicadores minerales antes de correr primera etapa
</commit_message>
<xml_diff>
--- a/docs/nomenclatura_variables_STATA.xlsx
+++ b/docs/nomenclatura_variables_STATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniandes-my.sharepoint.com/personal/jc_alfonso2004_uniandes_edu_co/Documents/PEG/PEG-mining-agriculture/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{C417AB08-1E28-4311-8367-541A348BB63C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E12BAA68-3467-4745-BB07-7E7179D1DA09}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{C417AB08-1E28-4311-8367-541A348BB63C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C650A738-DA16-4A30-A674-B8AE710E9AD7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1A4B0928-5C6E-441C-B24F-6FC110634DAB}"/>
+    <workbookView xWindow="14670" yWindow="1620" windowWidth="14130" windowHeight="13260" xr2:uid="{1A4B0928-5C6E-441C-B24F-6FC110634DAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
   <si>
     <t>Info</t>
   </si>
@@ -138,6 +138,45 @@
   </si>
   <si>
     <t>Evitar caracteres especiales como "ñ" o tildes</t>
+  </si>
+  <si>
+    <t>titu</t>
+  </si>
+  <si>
+    <t>Mine</t>
+  </si>
+  <si>
+    <t>Oro</t>
+  </si>
+  <si>
+    <t>fArSol</t>
+  </si>
+  <si>
+    <t>SArSol</t>
+  </si>
+  <si>
+    <t>mGrn</t>
+  </si>
+  <si>
+    <t>mOtr</t>
+  </si>
+  <si>
+    <t>concepto_sujeto_medicion_detalle_unidades</t>
+  </si>
+  <si>
+    <t>sujeto: 6</t>
+  </si>
+  <si>
+    <t>medicion: 6</t>
+  </si>
+  <si>
+    <t>concepto: 8</t>
+  </si>
+  <si>
+    <t>detalle: 4</t>
+  </si>
+  <si>
+    <t>unidades: 4</t>
   </si>
 </sst>
 </file>
@@ -509,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D129D89A-50F3-40F3-A3F5-8F31EBF8A9DF}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -517,12 +556,17 @@
     <col min="3" max="3" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -532,40 +576,64 @@
       <c r="C4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
       <c r="B8">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -573,15 +641,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -589,15 +663,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -605,7 +685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -613,7 +693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>

</xml_diff>